<commit_message>
Filter invitations to exclude entries with empty Email or Name fields; update user login ID in SharePoint script
</commit_message>
<xml_diff>
--- a/Input Data/invitations.xlsx
+++ b/Input Data/invitations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DakotaRuhl\Documents\PS-DR\Input Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E63E2F2-169F-4F7C-8D97-1C554C95DEF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CAFDD62-0C08-434A-9D3C-A132C898C91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
   </bookViews>
   <sheets>
     <sheet name="invitations" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>Source Data Reference:</t>
   </si>
@@ -88,107 +88,35 @@
     <t>Sponsor</t>
   </si>
   <si>
-    <t>aadeyefa@nisource.com (Ayo Adeyefa), gfields@nisource.com (Gregory Fields), twulkow@nisource.com (Tyler Wulkow), drose@nisource.com (David Rose), mluhrs@nisource.com (Michael Luhrs), DDouglas@nisource.com (Daniel L Douglas), dtwilliamson@nisource.com (Daniel T Williamson), mcroucher@nisource.com (Matthew Croucher), tmrodgers@nisource.com (Todd M Rodgers), pdentremont@nisource.com (Patrick Michael D'Entremont), cpatel@nisource.com (Chirag Patel), AGale@nisource.com (Adam Douglas Gale), jlionberg@nisource.com (Jason Lionberg), SHolcomb@nisource.com (Stephen Holcomb), aschroeder@nisource.com (Alan Schroeder)</t>
-  </si>
-  <si>
-    <t>Ayo Adeyefa</t>
-  </si>
-  <si>
-    <t>aadeyefa@nisource.com</t>
-  </si>
-  <si>
-    <t>Gregory Fields</t>
-  </si>
-  <si>
-    <t>gfields@nisource.com</t>
-  </si>
-  <si>
-    <t>Tyler Wulkow</t>
-  </si>
-  <si>
-    <t>twulkow@nisource.com</t>
-  </si>
-  <si>
-    <t>David Rose</t>
-  </si>
-  <si>
-    <t>drose@nisource.com</t>
-  </si>
-  <si>
-    <t>Michael Luhrs</t>
-  </si>
-  <si>
-    <t>mluhrs@nisource.com</t>
-  </si>
-  <si>
-    <t>Daniel L Douglas</t>
-  </si>
-  <si>
-    <t>DDouglas@nisource.com</t>
-  </si>
-  <si>
-    <t>Daniel T Williamson</t>
-  </si>
-  <si>
-    <t>dtwilliamson@nisource.com</t>
-  </si>
-  <si>
-    <t>Matthew Croucher</t>
-  </si>
-  <si>
-    <t>mcroucher@nisource.com</t>
-  </si>
-  <si>
-    <t>Todd M Rodgers</t>
-  </si>
-  <si>
-    <t>tmrodgers@nisource.com</t>
-  </si>
-  <si>
-    <t>Patrick Michael D'Entremont</t>
-  </si>
-  <si>
-    <t>pdentremont@nisource.com</t>
-  </si>
-  <si>
-    <t>Chirag Patel</t>
-  </si>
-  <si>
-    <t>cpatel@nisource.com</t>
-  </si>
-  <si>
-    <t>Adam Douglas Gale</t>
-  </si>
-  <si>
-    <t>AGale@nisource.com</t>
-  </si>
-  <si>
-    <t>Jason Lionberg</t>
-  </si>
-  <si>
-    <t>jlionberg@nisource.com</t>
-  </si>
-  <si>
-    <t>Stephen Holcomb</t>
-  </si>
-  <si>
-    <t>SHolcomb@nisource.com</t>
-  </si>
-  <si>
-    <t>Alan Schroeder</t>
-  </si>
-  <si>
-    <t>aschroeder@nisource.com</t>
+    <t>mquinones@loi-engineers.com (M Quinones), tmartin@loi-engineers.com (t martin), jdcordova@loi-engineers.com (j dcordova), hfpariente@loi-engineers.com (h fpariente) imontgomery@loi-engineers.com (I montgomery), venciso@loi-engineers.com (v enciso)</t>
   </si>
   <si>
     <t>cmaness@erock.com</t>
+  </si>
+  <si>
+    <t>gallend@bv.com</t>
+  </si>
+  <si>
+    <t>Nicholas Galle</t>
+  </si>
+  <si>
+    <t>EKolar@nisource.com</t>
+  </si>
+  <si>
+    <t>Edward Kolar</t>
+  </si>
+  <si>
+    <t>BBurns@nisource.com</t>
+  </si>
+  <si>
+    <t>Bryan Burns</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -319,14 +247,6 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -635,7 +555,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="43">
+  <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -678,17 +598,15 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="43">
+  <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -722,7 +640,6 @@
     <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -744,10 +661,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1067,12 +980,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D2F8AA2-E404-466B-9250-8D55F8A74E0E}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1087,140 +1000,157 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
+      <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>15</v>
+      <c r="A4" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>16</v>
       </c>
+      <c r="C4" s="3"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>22</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" t="s">
-        <v>24</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" t="s">
-        <v>26</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" t="s">
-        <v>28</v>
-      </c>
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" t="s">
-        <v>30</v>
-      </c>
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" t="s">
-        <v>32</v>
-      </c>
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" t="s">
-        <v>34</v>
-      </c>
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" t="s">
-        <v>36</v>
-      </c>
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" t="s">
-        <v>38</v>
-      </c>
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" t="s">
-        <v>40</v>
-      </c>
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1" xr:uid="{B72EC9D8-A683-4772-A03F-01331305709B}"/>
-    <hyperlink ref="B7" r:id="rId2" xr:uid="{28DCDCFF-BF58-4039-AE97-BD3B6441EF54}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88E9F234-5C3E-480D-ABE7-961177B0E2E5}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
@@ -1264,17 +1194,17 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="str" cm="1">
-        <f t="array" ref="A4:B18">_xlfn.LET(
+        <f t="array" ref="A4:B8">_xlfn.LET(
     _xlpm.source, E2,
     _xlpm.entries, TRANSPOSE(_xlfn.TEXTSPLIT(_xlpm.source, ", ")),
     _xlpm.names, _xlfn.MAP(_xlpm.entries, _xlfn.LAMBDA(_xlpm.e, TRIM(MID(_xlpm.e, FIND("(", _xlpm.e)+1, FIND(")", _xlpm.e)-FIND("(", _xlpm.e)-1)))),
     _xlpm.emails, _xlfn.MAP(_xlpm.entries, _xlfn.LAMBDA(_xlpm.e, TRIM(LEFT(_xlpm.e, FIND(" (", _xlpm.e)-1)))),
     _xlfn.HSTACK(_xlpm.names, _xlpm.emails)
 )</f>
-        <v>Ayo Adeyefa</v>
+        <v>M Quinones</v>
       </c>
       <c r="B4" t="str">
-        <v>aadeyefa@nisource.com</v>
+        <v>mquinones@loi-engineers.com</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
@@ -1282,115 +1212,39 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
-        <v>Gregory Fields</v>
+        <v>t martin</v>
       </c>
       <c r="B5" t="str">
-        <v>gfields@nisource.com</v>
+        <v>tmartin@loi-engineers.com</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
-        <v>Tyler Wulkow</v>
+        <v>j dcordova</v>
       </c>
       <c r="B6" t="str">
-        <v>twulkow@nisource.com</v>
+        <v>jdcordova@loi-engineers.com</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
-        <v>David Rose</v>
+        <v>h fpariente</v>
       </c>
       <c r="B7" t="str">
-        <v>drose@nisource.com</v>
-      </c>
-      <c r="E7" s="5"/>
+        <v>hfpariente@loi-engineers.com</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
-        <v>Michael Luhrs</v>
+        <v>v enciso</v>
       </c>
       <c r="B8" t="str">
-        <v>mluhrs@nisource.com</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="str">
-        <v>Daniel L Douglas</v>
-      </c>
-      <c r="B9" t="str">
-        <v>DDouglas@nisource.com</v>
+        <v>venciso@loi-engineers.com</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="str">
-        <v>Daniel T Williamson</v>
-      </c>
-      <c r="B10" t="str">
-        <v>dtwilliamson@nisource.com</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="str">
-        <v>Matthew Croucher</v>
-      </c>
-      <c r="B11" t="str">
-        <v>mcroucher@nisource.com</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="str">
-        <v>Todd M Rodgers</v>
-      </c>
-      <c r="B12" t="str">
-        <v>tmrodgers@nisource.com</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="str">
-        <v>Patrick Michael D'Entremont</v>
-      </c>
-      <c r="B13" t="str">
-        <v>pdentremont@nisource.com</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="str">
-        <v>Chirag Patel</v>
-      </c>
-      <c r="B14" t="str">
-        <v>cpatel@nisource.com</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="str">
-        <v>Adam Douglas Gale</v>
-      </c>
-      <c r="B15" t="str">
-        <v>AGale@nisource.com</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="str">
-        <v>Jason Lionberg</v>
-      </c>
-      <c r="B16" t="str">
-        <v>jlionberg@nisource.com</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="str">
-        <v>Stephen Holcomb</v>
-      </c>
-      <c r="B17" t="str">
-        <v>SHolcomb@nisource.com</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="str">
-        <v>Alan Schroeder</v>
-      </c>
-      <c r="B18" t="str">
-        <v>aschroeder@nisource.com</v>
+      <c r="E10" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor code structure for improved readability and maintainability. Created security groups creation script
</commit_message>
<xml_diff>
--- a/Input Data/invitations.xlsx
+++ b/Input Data/invitations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DakotaRuhl\Documents\PS-DR\Input Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CAFDD62-0C08-434A-9D3C-A132C898C91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2626DA30-A2F4-4359-BF1A-D794E557E931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t>Source Data Reference:</t>
   </si>
@@ -94,22 +94,10 @@
     <t>cmaness@erock.com</t>
   </si>
   <si>
-    <t>gallend@bv.com</t>
-  </si>
-  <si>
-    <t>Nicholas Galle</t>
-  </si>
-  <si>
-    <t>EKolar@nisource.com</t>
-  </si>
-  <si>
-    <t>Edward Kolar</t>
-  </si>
-  <si>
-    <t>BBurns@nisource.com</t>
-  </si>
-  <si>
-    <t>Bryan Burns</t>
+    <t>kmperes@nisource.com</t>
+  </si>
+  <si>
+    <t>Kevin Peres</t>
   </si>
 </sst>
 </file>
@@ -604,7 +592,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1003,29 +991,21 @@
       <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>14</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
       <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1129,18 +1109,12 @@
       <c r="C24" s="3"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
       <c r="C25" s="3"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
       <c r="C26" s="3"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
       <c r="C27" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add new PowerShell scripts for user and group reporting
- Created Test-UserSharePointGroupRemoval.ps1 to check user membership in SharePoint groups.
- Added AllDistributionGroupMembers.ps1 to export all distribution groups and their members to CSV.
- Introduced ArchiveMailboxSizeandStatus.ps1 for reporting on archive mailbox sizes and statuses.
- Implemented Microsoft365UserInfo.ps1 to gather user information from Azure AD.
- Developed OneDriveUsersStorageSizeReport.ps1 to report on OneDrive storage usage.
- Created Report-UserPasswordChanges&MFA.ps1 to report on user password changes and MFA status.
- Added menu.ps1 for a PowerShell TUI script launcher with enhanced logging.
- Generated initial log file for Launcher-Reports.
</commit_message>
<xml_diff>
--- a/Input Data/invitations.xlsx
+++ b/Input Data/invitations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DakotaRuhl\Documents\PS-DR\Input Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2626DA30-A2F4-4359-BF1A-D794E557E931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45855B75-DE88-41BC-933D-EF75A93B564A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>Source Data Reference:</t>
   </si>
@@ -88,16 +88,28 @@
     <t>Sponsor</t>
   </si>
   <si>
-    <t>mquinones@loi-engineers.com (M Quinones), tmartin@loi-engineers.com (t martin), jdcordova@loi-engineers.com (j dcordova), hfpariente@loi-engineers.com (h fpariente) imontgomery@loi-engineers.com (I montgomery), venciso@loi-engineers.com (v enciso)</t>
-  </si>
-  <si>
-    <t>cmaness@erock.com</t>
-  </si>
-  <si>
-    <t>kmperes@nisource.com</t>
-  </si>
-  <si>
-    <t>Kevin Peres</t>
+    <t>Jason Bickel Jason.Bickel@strategyeng.com (Jason Bickel), tim.collins@strategyeng.com (Tim Collins), Ronnie.Stuart@StrategyEng.com (Ronnie Stuart)</t>
+  </si>
+  <si>
+    <t>Jason Bickel</t>
+  </si>
+  <si>
+    <t>Tim Collins</t>
+  </si>
+  <si>
+    <t>tim.collins@strategyeng.com</t>
+  </si>
+  <si>
+    <t>Ronnie Stuart</t>
+  </si>
+  <si>
+    <t>Ronnie.Stuart@StrategyEng.com</t>
+  </si>
+  <si>
+    <t>arendon@erock.com</t>
+  </si>
+  <si>
+    <t>Jason.Bickel@strategyeng.com</t>
   </si>
 </sst>
 </file>
@@ -972,7 +984,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -989,23 +1001,31 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
       <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="C4" s="3"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1124,11 +1144,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88E9F234-5C3E-480D-ABE7-961177B0E2E5}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="59.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="66.7109375" customWidth="1"/>
   </cols>
@@ -1168,17 +1188,17 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="str" cm="1">
-        <f t="array" ref="A4:B8">_xlfn.LET(
+        <f t="array" ref="A4:B6">_xlfn.LET(
     _xlpm.source, E2,
     _xlpm.entries, TRANSPOSE(_xlfn.TEXTSPLIT(_xlpm.source, ", ")),
     _xlpm.names, _xlfn.MAP(_xlpm.entries, _xlfn.LAMBDA(_xlpm.e, TRIM(MID(_xlpm.e, FIND("(", _xlpm.e)+1, FIND(")", _xlpm.e)-FIND("(", _xlpm.e)-1)))),
     _xlpm.emails, _xlfn.MAP(_xlpm.entries, _xlfn.LAMBDA(_xlpm.e, TRIM(LEFT(_xlpm.e, FIND(" (", _xlpm.e)-1)))),
     _xlfn.HSTACK(_xlpm.names, _xlpm.emails)
 )</f>
-        <v>M Quinones</v>
+        <v>Jason Bickel</v>
       </c>
       <c r="B4" t="str">
-        <v>mquinones@loi-engineers.com</v>
+        <v>Jason Bickel Jason.Bickel@strategyeng.com</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
@@ -1186,38 +1206,22 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
-        <v>t martin</v>
+        <v>Tim Collins</v>
       </c>
       <c r="B5" t="str">
-        <v>tmartin@loi-engineers.com</v>
+        <v>tim.collins@strategyeng.com</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
-        <v>j dcordova</v>
+        <v>Ronnie Stuart</v>
       </c>
       <c r="B6" t="str">
-        <v>jdcordova@loi-engineers.com</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="str">
-        <v>h fpariente</v>
-      </c>
-      <c r="B7" t="str">
-        <v>hfpariente@loi-engineers.com</v>
+        <v>Ronnie.Stuart@StrategyEng.com</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="str">
-        <v>v enciso</v>
-      </c>
-      <c r="B8" t="str">
-        <v>venciso@loi-engineers.com</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E10" t="s">
+      <c r="E8" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add logs and backup configurations for Teams External Domains AllowList updates
- Created log files for two separate runs of the Teams External Domains AllowList process, capturing details such as the number of candidate domains, current allowed domains, and planned changes.
- Backed up the current federation configuration before making changes, ensuring that both the 162027 and 163930 timestamps are preserved for future reference.
- The backup JSON files include detailed lists of allowed domains and their configurations, maintaining consistency across updates.
</commit_message>
<xml_diff>
--- a/Input Data/invitations.xlsx
+++ b/Input Data/invitations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DakotaRuhl\Documents\PS-DR\Input Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45855B75-DE88-41BC-933D-EF75A93B564A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6F32A5-2569-4A95-AEE8-AF3F7C546D75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
   </bookViews>
   <sheets>
     <sheet name="invitations" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t>Source Data Reference:</t>
   </si>
@@ -91,25 +91,13 @@
     <t>Jason Bickel Jason.Bickel@strategyeng.com (Jason Bickel), tim.collins@strategyeng.com (Tim Collins), Ronnie.Stuart@StrategyEng.com (Ronnie Stuart)</t>
   </si>
   <si>
-    <t>Jason Bickel</t>
-  </si>
-  <si>
-    <t>Tim Collins</t>
-  </si>
-  <si>
-    <t>tim.collins@strategyeng.com</t>
-  </si>
-  <si>
-    <t>Ronnie Stuart</t>
-  </si>
-  <si>
-    <t>Ronnie.Stuart@StrategyEng.com</t>
-  </si>
-  <si>
-    <t>arendon@erock.com</t>
-  </si>
-  <si>
-    <t>Jason.Bickel@strategyeng.com</t>
+    <t>cmaness@erock.com</t>
+  </si>
+  <si>
+    <t>Edward Murtagh</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> emurtagh@nisource.com</t>
   </si>
 </sst>
 </file>
@@ -599,12 +587,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1001,31 +988,23 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>16</v>
-      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
       <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update guest invitation data, modify storage usage report script, and add group membership management script
- Updated GuestInviteResults.csv with new guest information.
- Modified VersionStorageUsageReport.ps1 to streamline report generation for the Titan library and added version trimming functionality.
- Introduced Entra-EnterpriseApps-CovertToGroup.ps1 for managing group memberships for enterprise applications, including user export and group creation.
- Added output files: AdobeAssignedUsers.csv, GroupMembershipResults.csv, and GroupMembershipFailures.csv to track user assignments and errors.
</commit_message>
<xml_diff>
--- a/Input Data/invitations.xlsx
+++ b/Input Data/invitations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DakotaRuhl\Documents\PS-DR\Input Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6F32A5-2569-4A95-AEE8-AF3F7C546D75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{982835D6-3CC3-4A2A-94B0-AC3B60A719DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
   </bookViews>
@@ -94,10 +94,10 @@
     <t>cmaness@erock.com</t>
   </si>
   <si>
-    <t>Edward Murtagh</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> emurtagh@nisource.com</t>
+    <t>FunkE@bv.com</t>
+  </si>
+  <si>
+    <t>Elizabeth Funk</t>
   </si>
 </sst>
 </file>
@@ -587,11 +587,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -988,10 +989,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>13</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Enhance guest invitation script with new parameters, update user removal logic, and modify storage usage report for improved functionality
</commit_message>
<xml_diff>
--- a/Input Data/invitations.xlsx
+++ b/Input Data/invitations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DakotaRuhl\Documents\PS-DR\Input Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{982835D6-3CC3-4A2A-94B0-AC3B60A719DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80BFE1C3-026D-46BF-871E-617A6DA4C1CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
   </bookViews>
   <sheets>
     <sheet name="invitations" sheetId="1" r:id="rId1"/>
@@ -91,13 +91,13 @@
     <t>Jason Bickel Jason.Bickel@strategyeng.com (Jason Bickel), tim.collins@strategyeng.com (Tim Collins), Ronnie.Stuart@StrategyEng.com (Ronnie Stuart)</t>
   </si>
   <si>
-    <t>cmaness@erock.com</t>
-  </si>
-  <si>
-    <t>FunkE@bv.com</t>
-  </si>
-  <si>
-    <t>Elizabeth Funk</t>
+    <t>Sabrina Dorsey</t>
+  </si>
+  <si>
+    <t>sabrina.dorsey@strategyeng.com</t>
+  </si>
+  <si>
+    <t>arendon@erock.com</t>
   </si>
 </sst>
 </file>
@@ -989,13 +989,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add new PowerShell scripts for guest invitations, OneDrive file copying, and password policy management; update CSV files for guest invites and copy results
</commit_message>
<xml_diff>
--- a/Input Data/invitations.xlsx
+++ b/Input Data/invitations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DakotaRuhl\Documents\PS-DR\Input Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80BFE1C3-026D-46BF-871E-617A6DA4C1CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE036C5-AC99-464C-AFDB-43D368F09BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4191656D-D1C9-4E47-95E8-944B227CEFF2}"/>
   </bookViews>
   <sheets>
     <sheet name="invitations" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>Source Data Reference:</t>
   </si>
@@ -88,23 +88,35 @@
     <t>Sponsor</t>
   </si>
   <si>
-    <t>Jason Bickel Jason.Bickel@strategyeng.com (Jason Bickel), tim.collins@strategyeng.com (Tim Collins), Ronnie.Stuart@StrategyEng.com (Ronnie Stuart)</t>
-  </si>
-  <si>
-    <t>Sabrina Dorsey</t>
-  </si>
-  <si>
-    <t>sabrina.dorsey@strategyeng.com</t>
-  </si>
-  <si>
-    <t>arendon@erock.com</t>
+    <t>karan.sharma@vrvision.ca (Karan Sharma), roni.cerga@vrvision.ca (Roni Cerga), david.tucciarone@vrvision.ca (David Tucciarone)</t>
+  </si>
+  <si>
+    <t>Karan Sharma</t>
+  </si>
+  <si>
+    <t>karan.sharma@vrvision.ca</t>
+  </si>
+  <si>
+    <t>Roni Cerga</t>
+  </si>
+  <si>
+    <t>roni.cerga@vrvision.ca</t>
+  </si>
+  <si>
+    <t>David Tucciarone</t>
+  </si>
+  <si>
+    <t>david.tucciarone@vrvision.ca</t>
+  </si>
+  <si>
+    <t>sabram@erock.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,6 +247,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -543,7 +563,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -586,15 +606,16 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -628,6 +649,7 @@
     <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -988,84 +1010,68 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
       <c r="C4" s="3"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
       <c r="C12" s="3"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
       <c r="C13" s="3"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
       <c r="C14" s="3"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
       <c r="C16" s="3"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1084,18 +1090,12 @@
       <c r="C19" s="3"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
       <c r="C20" s="3"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
       <c r="C21" s="3"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
       <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1118,19 +1118,22 @@
       <c r="C27" s="3"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{150C82F7-4BAD-4762-989C-74DA79DEB6BF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88E9F234-5C3E-480D-ABE7-961177B0E2E5}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="59.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="66.7109375" customWidth="1"/>
+    <col min="5" max="5" width="38.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1169,41 +1172,43 @@
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="str" cm="1">
         <f t="array" ref="A4:B6">_xlfn.LET(
-    _xlpm.source, E2,
-    _xlpm.entries, TRANSPOSE(_xlfn.TEXTSPLIT(_xlpm.source, ", ")),
+    _xlpm.source,E2,
+    _xlpm.entries, TRANSPOSE(_xlfn.TEXTSPLIT( _xlpm.source, ", ")),
     _xlpm.names, _xlfn.MAP(_xlpm.entries, _xlfn.LAMBDA(_xlpm.e, TRIM(MID(_xlpm.e, FIND("(", _xlpm.e)+1, FIND(")", _xlpm.e)-FIND("(", _xlpm.e)-1)))),
     _xlpm.emails, _xlfn.MAP(_xlpm.entries, _xlfn.LAMBDA(_xlpm.e, TRIM(LEFT(_xlpm.e, FIND(" (", _xlpm.e)-1)))),
     _xlfn.HSTACK(_xlpm.names, _xlpm.emails)
 )</f>
-        <v>Jason Bickel</v>
+        <v>Karan Sharma</v>
       </c>
       <c r="B4" t="str">
-        <v>Jason Bickel Jason.Bickel@strategyeng.com</v>
+        <v>karan.sharma@vrvision.ca</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
       </c>
+      <c r="E4" s="4"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
-        <v>Tim Collins</v>
+        <v>Roni Cerga</v>
       </c>
       <c r="B5" t="str">
-        <v>tim.collins@strategyeng.com</v>
+        <v>roni.cerga@vrvision.ca</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
-        <v>Ronnie Stuart</v>
+        <v>David Tucciarone</v>
       </c>
       <c r="B6" t="str">
-        <v>Ronnie.Stuart@StrategyEng.com</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E8" t="s">
-        <v>10</v>
-      </c>
+        <v>david.tucciarone@vrvision.ca</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E11" s="4"/>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E17" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>